<commit_message>
feat: Add report generation for desincorporaciones with ExcelJS
- Implemented a new method `generarReporte` in `desincorporacionesService.js` to generate a report based on desincorporacion data.
- The report is created using an Excel template and populated with relevant data including dependencies, responsible personnel, and associated bienes.
- Added logic to handle dynamic row duplication in the Excel sheet based on the number of bienes.
- Introduced a new Excel template `formato_desincorporacion.xlsx` for the report format.
- Updated existing Excel template `formato_inventario.xlsx` to reflect changes.

Co-authored-by: zapata888 <zapata888@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/server/src/templates/formato_inventario.xlsx
+++ b/server/src/templates/formato_inventario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usuario\Documents\Luisongo\Trayecto III\Aprendiendo Node.js\SIGADBP\server\src\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5425D61-B487-4D23-B691-1AA1933A8E5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22EF3629-3233-401E-8FEB-E32810EDAF36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9885C519-7CCA-4CFD-8609-2B5C3A63C552}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>N°</t>
   </si>
@@ -107,6 +107,9 @@
   </si>
   <si>
     <t>PAG:</t>
+  </si>
+  <si>
+    <t>FIRMA Y SELLO:</t>
   </si>
 </sst>
 </file>
@@ -176,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -191,6 +194,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -200,12 +210,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -588,85 +594,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="8"/>
+      <c r="A1" s="11"/>
       <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
       <c r="F1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
+      <c r="A2" s="11"/>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
+      <c r="A3" s="11"/>
       <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7" t="s">
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="10"/>
     </row>
     <row r="6" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6" t="s">
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
     </row>
     <row r="7" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6" t="s">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="6"/>
+      <c r="E7" s="9"/>
       <c r="F7" s="5" t="s">
         <v>16</v>
       </c>
@@ -852,47 +858,62 @@
       <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9" t="s">
+      <c r="A29" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
     </row>
     <row r="30" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11" t="s">
+      <c r="B30" s="8"/>
+      <c r="C30" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11" t="s">
+      <c r="D30" s="8"/>
+      <c r="E30" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F30" s="11"/>
+      <c r="F30" s="8"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-    </row>
-    <row r="32" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" ht="74.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F32" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="C1:E3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="C32:D32"/>
     <mergeCell ref="E32:F32"/>
@@ -903,15 +924,6 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="E30:F30"/>
     <mergeCell ref="E31:F31"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="C1:E3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A5:E5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>